<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-08 16:06
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
+++ b/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-05 14:39</t>
+          <t>2026-05-08 16:05</t>
         </is>
       </c>
     </row>
@@ -595,10 +595,10 @@
         <v>2</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0</v>
@@ -607,7 +607,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
     </row>
     <row r="6">
@@ -628,10 +628,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>0</v>
@@ -640,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
     </row>
     <row r="7">
@@ -661,10 +661,10 @@
         <v>2</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0</v>
@@ -673,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
     </row>
     <row r="8">
@@ -694,10 +694,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
       <c r="G8" s="10" t="n">
         <v>0</v>
@@ -706,7 +706,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>15000</v>
+        <v>14550</v>
       </c>
     </row>
     <row r="9">
@@ -727,10 +727,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0</v>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
     </row>
     <row r="10">
@@ -760,19 +760,19 @@
         <v>1</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>7500</v>
+        <v>7275</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>3750</v>
+        <v>3638</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>11250</v>
+        <v>10913</v>
       </c>
     </row>
     <row r="11">
@@ -793,19 +793,19 @@
         <v>1</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3750</v>
+        <v>3412</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>11250</v>
+        <v>10237</v>
       </c>
     </row>
     <row r="12">
@@ -826,10 +826,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G12" s="10" t="n">
         <v>0</v>
@@ -838,7 +838,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
     </row>
     <row r="13">
@@ -859,10 +859,10 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>0</v>
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
     </row>
     <row r="14">
@@ -892,10 +892,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>0</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
     </row>
     <row r="15">
@@ -925,19 +925,19 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3750</v>
+        <v>3412</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>11250</v>
+        <v>10237</v>
       </c>
     </row>
     <row r="16">
@@ -958,19 +958,19 @@
         <v>2</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>20000</v>
+        <v>18200</v>
       </c>
     </row>
     <row r="17">
@@ -991,10 +991,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
     </row>
     <row r="18">
@@ -1024,19 +1024,19 @@
         <v>1</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="19">
@@ -1057,19 +1057,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="20">
@@ -1090,19 +1090,19 @@
         <v>1</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="21">
@@ -1123,19 +1123,19 @@
         <v>2</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>20000</v>
+        <v>18200</v>
       </c>
     </row>
     <row r="22">
@@ -1156,10 +1156,10 @@
         <v>2</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G22" s="10" t="n">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
     </row>
     <row r="23">
@@ -1189,19 +1189,19 @@
         <v>1</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="24">
@@ -1222,19 +1222,19 @@
         <v>2</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>20000</v>
+        <v>18200</v>
       </c>
     </row>
     <row r="25">
@@ -1255,19 +1255,19 @@
         <v>3</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>24000</v>
+        <v>21840</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>28000</v>
+        <v>25480</v>
       </c>
     </row>
     <row r="26">
@@ -1288,10 +1288,10 @@
         <v>1</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
     </row>
     <row r="27">
@@ -1321,19 +1321,19 @@
         <v>1</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="28">
@@ -1354,10 +1354,10 @@
         <v>3</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>24000</v>
+        <v>21840</v>
       </c>
       <c r="G28" s="10" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>24000</v>
+        <v>21840</v>
       </c>
     </row>
     <row r="29">
@@ -1387,10 +1387,10 @@
         <v>2</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>0</v>
@@ -1399,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
     </row>
     <row r="30">
@@ -1420,19 +1420,19 @@
         <v>1</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="31">
@@ -1453,19 +1453,19 @@
         <v>3</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>24000</v>
+        <v>21840</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>28000</v>
+        <v>25480</v>
       </c>
     </row>
     <row r="32">
@@ -1486,19 +1486,19 @@
         <v>1</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="33">
@@ -1519,10 +1519,10 @@
         <v>1</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>0</v>
@@ -1531,7 +1531,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
     </row>
     <row r="34">
@@ -1552,10 +1552,10 @@
         <v>2</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
       <c r="G34" s="10" t="n">
         <v>0</v>
@@ -1564,7 +1564,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>16000</v>
+        <v>14560</v>
       </c>
     </row>
     <row r="35">
@@ -1585,19 +1585,19 @@
         <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>8000</v>
+        <v>7280</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>4000</v>
+        <v>3640</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>12000</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="36">
@@ -1618,10 +1618,10 @@
         <v>2</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>15000</v>
+        <v>13650</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>15000</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="37">
@@ -1651,19 +1651,19 @@
         <v>1</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>3750</v>
+        <v>3412</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>11250</v>
+        <v>10237</v>
       </c>
     </row>
     <row r="38">
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="G38" s="10" t="n">
         <v>0</v>
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
     </row>
     <row r="39">
@@ -1717,19 +1717,19 @@
         <v>3</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>22500</v>
+        <v>20475</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3750</v>
+        <v>3412</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>26250</v>
+        <v>23887</v>
       </c>
     </row>
     <row r="40">
@@ -1750,10 +1750,10 @@
         <v>2</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>7500</v>
+        <v>6825</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>15000</v>
+        <v>13650</v>
       </c>
       <c r="G40" s="10" t="n">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="10" t="n">
-        <v>15000</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="41">
@@ -1783,10 +1783,10 @@
         <v>2</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="42">
@@ -1816,19 +1816,19 @@
         <v>2</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>3750</v>
+        <v>3300</v>
       </c>
       <c r="H42" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="10" t="n">
-        <v>18750</v>
+        <v>16500</v>
       </c>
     </row>
     <row r="43">
@@ -1849,10 +1849,10 @@
         <v>2</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="44">
@@ -1882,10 +1882,10 @@
         <v>2</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G44" s="10" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="45">
@@ -1915,10 +1915,10 @@
         <v>2</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="46">
@@ -1948,10 +1948,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G46" s="10" t="n">
         <v>0</v>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="47">
@@ -1981,10 +1981,10 @@
         <v>1</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>0</v>
@@ -1993,7 +1993,7 @@
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="48">
@@ -2014,10 +2014,10 @@
         <v>1</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G48" s="10" t="n">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="49">
@@ -2047,10 +2047,10 @@
         <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>0</v>
@@ -2059,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="50">
@@ -2080,19 +2080,19 @@
         <v>1</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>3750</v>
+        <v>3300</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>11250</v>
+        <v>9900</v>
       </c>
     </row>
     <row r="51">
@@ -2113,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>0</v>
@@ -2125,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="52">
@@ -2146,10 +2146,10 @@
         <v>2</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G52" s="10" t="n">
         <v>0</v>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="53">
@@ -2179,10 +2179,10 @@
         <v>2</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>0</v>
@@ -2191,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="54">
@@ -2212,10 +2212,10 @@
         <v>1</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G54" s="10" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="55">
@@ -2245,10 +2245,10 @@
         <v>1</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="56">
@@ -2278,10 +2278,10 @@
         <v>2</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="F56" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>15000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="57">
@@ -2311,19 +2311,19 @@
         <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G57" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="H57" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>15000</v>
+        <v>13100</v>
       </c>
     </row>
     <row r="58">
@@ -2344,19 +2344,19 @@
         <v>1</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="H58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I58" s="10" t="n">
-        <v>15000</v>
+        <v>13100</v>
       </c>
     </row>
     <row r="59">
@@ -2377,19 +2377,19 @@
         <v>1</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>7500</v>
+        <v>6600</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>15000</v>
+        <v>13100</v>
       </c>
     </row>
     <row r="60">
@@ -2410,19 +2410,19 @@
         <v>1</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H60" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I60" s="10" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="61">
@@ -2443,19 +2443,19 @@
         <v>2</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>22500</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="62">
@@ -2476,19 +2476,19 @@
         <v>1</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="10" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="63">
@@ -2509,19 +2509,19 @@
         <v>1</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="64">
@@ -2542,19 +2542,19 @@
         <v>2</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>15000</v>
+        <v>14000</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H64" s="10" t="n">
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="I64" s="10" t="n">
-        <v>26250</v>
+        <v>17250</v>
       </c>
     </row>
     <row r="65">
@@ -2575,19 +2575,19 @@
         <v>1</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="66">
@@ -2608,19 +2608,19 @@
         <v>1</v>
       </c>
       <c r="E66" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="10" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="67">
@@ -2641,19 +2641,19 @@
         <v>1</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G67" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H67" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="68">
@@ -2674,19 +2674,19 @@
         <v>0</v>
       </c>
       <c r="E68" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F68" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H68" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I68" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="69">
@@ -2707,19 +2707,19 @@
         <v>1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="70">
@@ -2740,10 +2740,10 @@
         <v>3</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F70" s="10" t="n">
-        <v>22500</v>
+        <v>19500</v>
       </c>
       <c r="G70" s="10" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         <v>0</v>
       </c>
       <c r="I70" s="10" t="n">
-        <v>22500</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="71">
@@ -2773,10 +2773,10 @@
         <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>0</v>
@@ -2785,7 +2785,7 @@
         <v>0</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="72">
@@ -2806,19 +2806,19 @@
         <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H72" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I72" s="10" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="73">
@@ -2839,19 +2839,19 @@
         <v>1</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F73" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G73" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H73" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="74">
@@ -2872,19 +2872,19 @@
         <v>1</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F74" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H74" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I74" s="10" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="75">
@@ -2905,19 +2905,19 @@
         <v>0</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F75" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G75" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H75" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="76">
@@ -2938,19 +2938,19 @@
         <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H76" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I76" s="10" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="77">
@@ -2971,19 +2971,19 @@
         <v>1</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G77" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="H77" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="78">
@@ -3004,19 +3004,19 @@
         <v>1</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I78" s="10" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="79">
@@ -3037,19 +3037,19 @@
         <v>1</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>7500</v>
+        <v>7378</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>7500</v>
+        <v>7378</v>
       </c>
       <c r="G79" s="7" t="n">
-        <v>3750</v>
+        <v>3689</v>
       </c>
       <c r="H79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>11250</v>
+        <v>11067</v>
       </c>
     </row>
     <row r="80">
@@ -3070,19 +3070,19 @@
         <v>1</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>7500</v>
+        <v>7378</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>7500</v>
+        <v>7378</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>3750</v>
+        <v>3689</v>
       </c>
       <c r="H80" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I80" s="10" t="n">
-        <v>11250</v>
+        <v>11067</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-08 18:17
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
+++ b/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08 17:39</t>
+          <t>2026-05-08 18:09</t>
         </is>
       </c>
     </row>
@@ -595,10 +595,10 @@
         <v>2</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0</v>
@@ -607,7 +607,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
     </row>
     <row r="6">
@@ -628,10 +628,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>0</v>
@@ -640,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
     </row>
     <row r="7">
@@ -661,10 +661,10 @@
         <v>2</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0</v>
@@ -673,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
     </row>
     <row r="8">
@@ -694,10 +694,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
       <c r="G8" s="10" t="n">
         <v>0</v>
@@ -706,7 +706,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>14550</v>
+        <v>14553.38</v>
       </c>
     </row>
     <row r="9">
@@ -727,10 +727,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0</v>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
     </row>
     <row r="10">
@@ -760,10 +760,10 @@
         <v>1</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>7275</v>
+        <v>7276.69</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>3638</v>
@@ -772,7 +772,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>10913</v>
+        <v>10914.69</v>
       </c>
     </row>
     <row r="11">
@@ -793,19 +793,19 @@
         <v>1</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3412</v>
+        <v>3425</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>10237</v>
+        <v>10274.81</v>
       </c>
     </row>
     <row r="12">
@@ -826,10 +826,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G12" s="10" t="n">
         <v>0</v>
@@ -838,7 +838,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
     </row>
     <row r="13">
@@ -859,10 +859,10 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>0</v>
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
     </row>
     <row r="14">
@@ -892,10 +892,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>0</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
     </row>
     <row r="15">
@@ -925,19 +925,19 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3412</v>
+        <v>3425</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>10237</v>
+        <v>10274.81</v>
       </c>
     </row>
     <row r="16">
@@ -958,19 +958,19 @@
         <v>2</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>18200</v>
+        <v>18265.94</v>
       </c>
     </row>
     <row r="17">
@@ -991,10 +991,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
     </row>
     <row r="18">
@@ -1024,19 +1024,19 @@
         <v>1</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="19">
@@ -1057,19 +1057,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="20">
@@ -1090,19 +1090,19 @@
         <v>1</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="21">
@@ -1123,19 +1123,19 @@
         <v>2</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>18200</v>
+        <v>18265.94</v>
       </c>
     </row>
     <row r="22">
@@ -1156,10 +1156,10 @@
         <v>2</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G22" s="10" t="n">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
     </row>
     <row r="23">
@@ -1189,19 +1189,19 @@
         <v>1</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="24">
@@ -1222,19 +1222,19 @@
         <v>2</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>18200</v>
+        <v>18265.94</v>
       </c>
     </row>
     <row r="25">
@@ -1255,19 +1255,19 @@
         <v>3</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>21840</v>
+        <v>21919.41</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>25480</v>
+        <v>25572.41</v>
       </c>
     </row>
     <row r="26">
@@ -1288,10 +1288,10 @@
         <v>1</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
     </row>
     <row r="27">
@@ -1321,19 +1321,19 @@
         <v>1</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="28">
@@ -1354,10 +1354,10 @@
         <v>3</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>21840</v>
+        <v>21919.41</v>
       </c>
       <c r="G28" s="10" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>21840</v>
+        <v>21919.41</v>
       </c>
     </row>
     <row r="29">
@@ -1387,10 +1387,10 @@
         <v>2</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>0</v>
@@ -1399,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
     </row>
     <row r="30">
@@ -1420,19 +1420,19 @@
         <v>1</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="31">
@@ -1453,19 +1453,19 @@
         <v>3</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>21840</v>
+        <v>21919.41</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>25480</v>
+        <v>25572.41</v>
       </c>
     </row>
     <row r="32">
@@ -1486,19 +1486,19 @@
         <v>1</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="33">
@@ -1519,10 +1519,10 @@
         <v>1</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>0</v>
@@ -1531,7 +1531,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
     </row>
     <row r="34">
@@ -1552,10 +1552,10 @@
         <v>2</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
       <c r="G34" s="10" t="n">
         <v>0</v>
@@ -1564,7 +1564,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>14560</v>
+        <v>14612.94</v>
       </c>
     </row>
     <row r="35">
@@ -1585,19 +1585,19 @@
         <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>7280</v>
+        <v>7306.47</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>3640</v>
+        <v>3653</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>10920</v>
+        <v>10959.47</v>
       </c>
     </row>
     <row r="36">
@@ -1618,10 +1618,10 @@
         <v>2</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>13650</v>
+        <v>13699.62</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>13650</v>
+        <v>13699.62</v>
       </c>
     </row>
     <row r="37">
@@ -1651,19 +1651,19 @@
         <v>1</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>3412</v>
+        <v>3425</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>10237</v>
+        <v>10274.81</v>
       </c>
     </row>
     <row r="38">
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="G38" s="10" t="n">
         <v>0</v>
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
     </row>
     <row r="39">
@@ -1717,19 +1717,19 @@
         <v>3</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>20475</v>
+        <v>20549.43</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3412</v>
+        <v>3425</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>23887</v>
+        <v>23974.43</v>
       </c>
     </row>
     <row r="40">
@@ -1750,10 +1750,10 @@
         <v>2</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>6825</v>
+        <v>6849.81</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>13650</v>
+        <v>13699.62</v>
       </c>
       <c r="G40" s="10" t="n">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="10" t="n">
-        <v>13650</v>
+        <v>13699.62</v>
       </c>
     </row>
     <row r="41">
@@ -1783,10 +1783,10 @@
         <v>2</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="42">
@@ -1816,19 +1816,19 @@
         <v>2</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>3300</v>
+        <v>3323</v>
       </c>
       <c r="H42" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="10" t="n">
-        <v>16500</v>
+        <v>16614.72</v>
       </c>
     </row>
     <row r="43">
@@ -1849,10 +1849,10 @@
         <v>2</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="44">
@@ -1882,10 +1882,10 @@
         <v>2</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G44" s="10" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="45">
@@ -1915,10 +1915,10 @@
         <v>2</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="46">
@@ -1948,10 +1948,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G46" s="10" t="n">
         <v>0</v>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="47">
@@ -1981,10 +1981,10 @@
         <v>1</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>0</v>
@@ -1993,7 +1993,7 @@
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="48">
@@ -2014,10 +2014,10 @@
         <v>1</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G48" s="10" t="n">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="49">
@@ -2047,10 +2047,10 @@
         <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>0</v>
@@ -2059,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="50">
@@ -2080,19 +2080,19 @@
         <v>1</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>3300</v>
+        <v>3323</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>9900</v>
+        <v>9968.860000000001</v>
       </c>
     </row>
     <row r="51">
@@ -2113,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>0</v>
@@ -2125,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="52">
@@ -2146,10 +2146,10 @@
         <v>2</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G52" s="10" t="n">
         <v>0</v>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="53">
@@ -2179,10 +2179,10 @@
         <v>2</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>0</v>
@@ -2191,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="54">
@@ -2212,10 +2212,10 @@
         <v>1</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G54" s="10" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="55">
@@ -2245,10 +2245,10 @@
         <v>1</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
     </row>
     <row r="56">
@@ -2278,10 +2278,10 @@
         <v>2</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>6600</v>
+        <v>6645.86</v>
       </c>
       <c r="F56" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>13200</v>
+        <v>13291.72</v>
       </c>
     </row>
     <row r="57">
@@ -2311,19 +2311,19 @@
         <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G57" s="7" t="n">
-        <v>6600</v>
+        <v>6645</v>
       </c>
       <c r="H57" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>13100</v>
+        <v>13191.17</v>
       </c>
     </row>
     <row r="58">
@@ -2344,19 +2344,19 @@
         <v>1</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>6600</v>
+        <v>6645</v>
       </c>
       <c r="H58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I58" s="10" t="n">
-        <v>13100</v>
+        <v>13191.17</v>
       </c>
     </row>
     <row r="59">
@@ -2377,19 +2377,19 @@
         <v>1</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>6600</v>
+        <v>6645</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>13100</v>
+        <v>13191.17</v>
       </c>
     </row>
     <row r="60">
@@ -2410,19 +2410,19 @@
         <v>1</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>3250</v>
+        <v>3273</v>
       </c>
       <c r="H60" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I60" s="10" t="n">
-        <v>9750</v>
+        <v>9819.17</v>
       </c>
     </row>
     <row r="61">
@@ -2443,19 +2443,19 @@
         <v>2</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>13000</v>
+        <v>13092.34</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>6500</v>
+        <v>6546</v>
       </c>
       <c r="H61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>19500</v>
+        <v>19638.34</v>
       </c>
     </row>
     <row r="62">
@@ -2476,19 +2476,19 @@
         <v>1</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>3250</v>
+        <v>3273</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="10" t="n">
-        <v>9750</v>
+        <v>9819.17</v>
       </c>
     </row>
     <row r="63">
@@ -2509,19 +2509,19 @@
         <v>1</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>3250</v>
+        <v>3273</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>9750</v>
+        <v>9819.17</v>
       </c>
     </row>
     <row r="64">
@@ -2542,19 +2542,19 @@
         <v>2</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>14000</v>
+        <v>14046</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>3250</v>
+        <v>3273</v>
       </c>
       <c r="H64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I64" s="10" t="n">
-        <v>17250</v>
+        <v>17319</v>
       </c>
     </row>
     <row r="65">
@@ -2575,19 +2575,19 @@
         <v>1</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>6500</v>
+        <v>6546.17</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>3250</v>
+        <v>3273</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>9750</v>
+        <v>9819.17</v>
       </c>
     </row>
     <row r="66">
@@ -3037,19 +3037,19 @@
         <v>1</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>7378</v>
+        <v>7432.03</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>7378</v>
+        <v>7432.03</v>
       </c>
       <c r="G79" s="7" t="n">
-        <v>3689</v>
+        <v>3716</v>
       </c>
       <c r="H79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>11067</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="80">
@@ -3070,19 +3070,19 @@
         <v>1</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>7378</v>
+        <v>7432.03</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>7378</v>
+        <v>7432.03</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>3689</v>
+        <v>3716</v>
       </c>
       <c r="H80" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I80" s="10" t="n">
-        <v>11067</v>
+        <v>11148.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-26 13:16
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
+++ b/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-26 13:09</t>
+          <t>2026-05-26 13:16</t>
         </is>
       </c>
     </row>
@@ -628,19 +628,19 @@
         <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="7">
@@ -661,19 +661,19 @@
         <v>1</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="8">
@@ -694,19 +694,19 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
     </row>
     <row r="9">
@@ -727,19 +727,19 @@
         <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>7432</v>
+        <v>6598</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>14864.03</v>
+        <v>13195.5</v>
       </c>
     </row>
     <row r="10">
@@ -760,19 +760,19 @@
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
     </row>
     <row r="11">
@@ -793,19 +793,19 @@
         <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
     </row>
     <row r="12">
@@ -826,19 +826,19 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="13">
@@ -859,19 +859,19 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="14">
@@ -892,19 +892,19 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="15">
@@ -925,19 +925,19 @@
         <v>2</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>7432</v>
+        <v>6598</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>22296.06</v>
+        <v>19793</v>
       </c>
     </row>
     <row r="16">
@@ -958,19 +958,19 @@
         <v>1</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="17">
@@ -991,19 +991,19 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="18">
@@ -1024,19 +1024,19 @@
         <v>1</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="19">
@@ -1057,19 +1057,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="20">
@@ -1090,19 +1090,19 @@
         <v>2</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>18580.06</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="21">
@@ -1123,19 +1123,19 @@
         <v>2</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>18580.06</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="22">
@@ -1156,19 +1156,19 @@
         <v>1</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="23">
@@ -1189,19 +1189,19 @@
         <v>1</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>11148.03</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="24">
@@ -1222,10 +1222,10 @@
         <v>2</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
       <c r="G24" s="10" t="n">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
     </row>
     <row r="25">
@@ -1255,19 +1255,19 @@
         <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>7432.03</v>
+        <v>6597.5</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>14864.06</v>
+        <v>13195</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>3716</v>
+        <v>3299</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>18580.06</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="26">
@@ -1288,19 +1288,19 @@
         <v>1</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>3661</v>
+        <v>3250</v>
       </c>
       <c r="H26" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>10983.2</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="27">
@@ -1321,10 +1321,10 @@
         <v>2</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>0</v>
@@ -1333,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="28">
@@ -1354,10 +1354,10 @@
         <v>1</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G28" s="10" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="29">
@@ -1387,19 +1387,19 @@
         <v>1</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3661</v>
+        <v>3250</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>10983.2</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="30">
@@ -1420,19 +1420,19 @@
         <v>1</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>3661</v>
+        <v>3250</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>10983.2</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="31">
@@ -1453,10 +1453,10 @@
         <v>1</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>0</v>
@@ -1465,7 +1465,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="32">
@@ -1486,19 +1486,19 @@
         <v>2</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>3661</v>
+        <v>3250</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>18305.4</v>
+        <v>16250</v>
       </c>
     </row>
     <row r="33">
@@ -1519,19 +1519,19 @@
         <v>2</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>7322</v>
+        <v>6500</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>21966.4</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="34">
@@ -1552,10 +1552,10 @@
         <v>1</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G34" s="10" t="n">
         <v>0</v>
@@ -1564,7 +1564,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="35">
@@ -1585,19 +1585,19 @@
         <v>2</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>7322</v>
+        <v>6500</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>21966.4</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="36">
@@ -1618,10 +1618,10 @@
         <v>1</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="37">
@@ -1651,10 +1651,10 @@
         <v>2</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G37" s="7" t="n">
         <v>0</v>
@@ -1663,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="38">
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G38" s="10" t="n">
         <v>0</v>
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="39">
@@ -1717,19 +1717,19 @@
         <v>2</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3661</v>
+        <v>3250</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>18305.4</v>
+        <v>16250</v>
       </c>
     </row>
     <row r="40">
@@ -1750,10 +1750,10 @@
         <v>1</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="G40" s="10" t="n">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="10" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="41">
@@ -1783,10 +1783,10 @@
         <v>2</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>7322.2</v>
+        <v>6500</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>14644.4</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="42">
@@ -1816,10 +1816,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G42" s="10" t="n">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="43">
@@ -1849,19 +1849,19 @@
         <v>2</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>18305.4</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="44">
@@ -1882,10 +1882,10 @@
         <v>2</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G44" s="10" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
     </row>
     <row r="45">
@@ -1915,10 +1915,10 @@
         <v>1</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="46">
@@ -1948,10 +1948,10 @@
         <v>2</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G46" s="10" t="n">
         <v>0</v>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
     </row>
     <row r="47">
@@ -1981,19 +1981,19 @@
         <v>2</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>18305.4</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="48">
@@ -2014,19 +2014,19 @@
         <v>2</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G48" s="10" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>18305.4</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="49">
@@ -2047,19 +2047,19 @@
         <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>10983.2</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="50">
@@ -2080,10 +2080,10 @@
         <v>2</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G50" s="10" t="n">
         <v>0</v>
@@ -2092,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
     </row>
     <row r="51">
@@ -2113,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>0</v>
@@ -2125,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="52">
@@ -2146,10 +2146,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G52" s="10" t="n">
         <v>0</v>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="53">
@@ -2179,19 +2179,19 @@
         <v>2</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>14644.4</v>
+        <v>13195</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>18305.4</v>
+        <v>16494</v>
       </c>
     </row>
     <row r="54">
@@ -2212,10 +2212,10 @@
         <v>3</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>21966.6</v>
+        <v>19792.5</v>
       </c>
       <c r="G54" s="10" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>21966.6</v>
+        <v>19792.5</v>
       </c>
     </row>
     <row r="55">
@@ -2245,10 +2245,10 @@
         <v>1</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="56">
@@ -2278,10 +2278,10 @@
         <v>1</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F56" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="57">
@@ -2311,10 +2311,10 @@
         <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>0</v>
@@ -2323,7 +2323,7 @@
         <v>0</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="58">
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G58" s="10" t="n">
         <v>0</v>
@@ -2356,7 +2356,7 @@
         <v>0</v>
       </c>
       <c r="I58" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="59">
@@ -2377,19 +2377,19 @@
         <v>1</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>3661</v>
+        <v>3299</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>10983.2</v>
+        <v>9896.5</v>
       </c>
     </row>
     <row r="60">
@@ -2410,10 +2410,10 @@
         <v>1</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
       <c r="G60" s="10" t="n">
         <v>0</v>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
       <c r="I60" s="10" t="n">
-        <v>7322.2</v>
+        <v>6597.5</v>
       </c>
     </row>
     <row r="61">
@@ -2443,19 +2443,19 @@
         <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="62">
@@ -2476,19 +2476,19 @@
         <v>2</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="10" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="63">
@@ -2509,19 +2509,19 @@
         <v>2</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="64">
@@ -2542,19 +2542,19 @@
         <v>1</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I64" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="65">
@@ -2575,19 +2575,19 @@
         <v>2</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="66">
@@ -2608,19 +2608,19 @@
         <v>1</v>
       </c>
       <c r="E66" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="67">
@@ -2641,10 +2641,10 @@
         <v>2</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>0</v>
@@ -2653,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
     </row>
     <row r="68">
@@ -2674,19 +2674,19 @@
         <v>2</v>
       </c>
       <c r="E68" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F68" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H68" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I68" s="10" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="69">
@@ -2707,19 +2707,19 @@
         <v>1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="70">
@@ -2740,10 +2740,10 @@
         <v>1</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F70" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G70" s="10" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         <v>0</v>
       </c>
       <c r="I70" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="71">
@@ -2773,10 +2773,10 @@
         <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>0</v>
@@ -2785,7 +2785,7 @@
         <v>0</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
     </row>
     <row r="72">
@@ -2806,10 +2806,10 @@
         <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G72" s="10" t="n">
         <v>0</v>
@@ -2818,7 +2818,7 @@
         <v>0</v>
       </c>
       <c r="I72" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="73">
@@ -2839,19 +2839,19 @@
         <v>1</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F73" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G73" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H73" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="74">
@@ -2872,19 +2872,19 @@
         <v>1</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F74" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H74" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I74" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="75">
@@ -2905,19 +2905,19 @@
         <v>1</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F75" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G75" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H75" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="76">
@@ -2938,10 +2938,10 @@
         <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G76" s="10" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="I76" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="77">
@@ -2971,19 +2971,19 @@
         <v>1</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G77" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H77" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="78">
@@ -3004,19 +3004,19 @@
         <v>1</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I78" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="79">
@@ -3037,19 +3037,19 @@
         <v>2</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G79" s="7" t="n">
-        <v>7322</v>
+        <v>6696</v>
       </c>
       <c r="H79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>21966.4</v>
+        <v>20088.92</v>
       </c>
     </row>
     <row r="80">
@@ -3070,10 +3070,10 @@
         <v>1</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>0</v>
@@ -3082,7 +3082,7 @@
         <v>0</v>
       </c>
       <c r="I80" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="81">
@@ -3103,19 +3103,19 @@
         <v>2</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G81" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H81" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="82">
@@ -3136,19 +3136,19 @@
         <v>1</v>
       </c>
       <c r="E82" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H82" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I82" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="83">
@@ -3169,10 +3169,10 @@
         <v>1</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F83" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G83" s="7" t="n">
         <v>0</v>
@@ -3181,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="84">
@@ -3202,19 +3202,19 @@
         <v>2</v>
       </c>
       <c r="E84" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H84" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I84" s="10" t="n">
-        <v>18305.4</v>
+        <v>16740.92</v>
       </c>
     </row>
     <row r="85">
@@ -3235,19 +3235,19 @@
         <v>1</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G85" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H85" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I85" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="86">
@@ -3268,10 +3268,10 @@
         <v>2</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>0</v>
@@ -3280,7 +3280,7 @@
         <v>0</v>
       </c>
       <c r="I86" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
     </row>
     <row r="87">
@@ -3301,19 +3301,19 @@
         <v>2</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F87" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G87" s="7" t="n">
-        <v>7322</v>
+        <v>6696</v>
       </c>
       <c r="H87" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>21966.4</v>
+        <v>20088.92</v>
       </c>
     </row>
     <row r="88">
@@ -3334,10 +3334,10 @@
         <v>2</v>
       </c>
       <c r="E88" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>0</v>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="I88" s="10" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
     </row>
     <row r="89">
@@ -3367,10 +3367,10 @@
         <v>1</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F89" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G89" s="7" t="n">
         <v>0</v>
@@ -3379,7 +3379,7 @@
         <v>0</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="90">
@@ -3400,10 +3400,10 @@
         <v>1</v>
       </c>
       <c r="E90" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>0</v>
@@ -3412,7 +3412,7 @@
         <v>0</v>
       </c>
       <c r="I90" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="91">
@@ -3433,19 +3433,19 @@
         <v>1</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F91" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G91" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H91" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I91" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="92">
@@ -3466,10 +3466,10 @@
         <v>1</v>
       </c>
       <c r="E92" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>0</v>
@@ -3478,7 +3478,7 @@
         <v>0</v>
       </c>
       <c r="I92" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="93">
@@ -3499,10 +3499,10 @@
         <v>1</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G93" s="7" t="n">
         <v>0</v>
@@ -3511,7 +3511,7 @@
         <v>0</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="94">
@@ -3532,10 +3532,10 @@
         <v>1</v>
       </c>
       <c r="E94" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F94" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>0</v>
@@ -3544,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="I94" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
     </row>
     <row r="95">
@@ -3565,19 +3565,19 @@
         <v>1</v>
       </c>
       <c r="E95" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F95" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G95" s="7" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H95" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="96">
@@ -3598,19 +3598,19 @@
         <v>1</v>
       </c>
       <c r="E96" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="G96" s="10" t="n">
-        <v>3661</v>
+        <v>3348</v>
       </c>
       <c r="H96" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I96" s="10" t="n">
-        <v>10983.2</v>
+        <v>10044.46</v>
       </c>
     </row>
     <row r="97">
@@ -3631,19 +3631,19 @@
         <v>2</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>7322.2</v>
+        <v>6696.46</v>
       </c>
       <c r="F97" s="7" t="n">
-        <v>14644.4</v>
+        <v>13392.92</v>
       </c>
       <c r="G97" s="7" t="n">
-        <v>7322</v>
+        <v>6696</v>
       </c>
       <c r="H97" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>21966.4</v>
+        <v>20088.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-26 13:20
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
+++ b/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-26 13:16</t>
+          <t>2026-05-26 13:20</t>
         </is>
       </c>
     </row>
@@ -628,19 +628,19 @@
         <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="7">
@@ -661,19 +661,19 @@
         <v>1</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="8">
@@ -694,19 +694,19 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
     </row>
     <row r="9">
@@ -727,19 +727,19 @@
         <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>6598</v>
+        <v>7432</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>13195.5</v>
+        <v>14864.03</v>
       </c>
     </row>
     <row r="10">
@@ -760,19 +760,19 @@
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
     </row>
     <row r="11">
@@ -793,19 +793,19 @@
         <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
     </row>
     <row r="12">
@@ -826,19 +826,19 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="13">
@@ -859,19 +859,19 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="14">
@@ -892,19 +892,19 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="15">
@@ -925,19 +925,19 @@
         <v>2</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6598</v>
+        <v>7432</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>19793</v>
+        <v>22296.06</v>
       </c>
     </row>
     <row r="16">
@@ -958,19 +958,19 @@
         <v>1</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="17">
@@ -991,19 +991,19 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="18">
@@ -1024,19 +1024,19 @@
         <v>1</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="19">
@@ -1057,19 +1057,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="20">
@@ -1090,19 +1090,19 @@
         <v>2</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>16494</v>
+        <v>18580.06</v>
       </c>
     </row>
     <row r="21">
@@ -1123,19 +1123,19 @@
         <v>2</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>16494</v>
+        <v>18580.06</v>
       </c>
     </row>
     <row r="22">
@@ -1156,19 +1156,19 @@
         <v>1</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="23">
@@ -1189,19 +1189,19 @@
         <v>1</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>9896.5</v>
+        <v>11148.03</v>
       </c>
     </row>
     <row r="24">
@@ -1222,10 +1222,10 @@
         <v>2</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G24" s="10" t="n">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
     </row>
     <row r="25">
@@ -1255,19 +1255,19 @@
         <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>16494</v>
+        <v>18580.06</v>
       </c>
     </row>
     <row r="26">
@@ -1288,19 +1288,19 @@
         <v>1</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>3250</v>
+        <v>3661</v>
       </c>
       <c r="H26" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>9750</v>
+        <v>10983.2</v>
       </c>
     </row>
     <row r="27">
@@ -1321,10 +1321,10 @@
         <v>2</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>0</v>
@@ -1333,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
     </row>
     <row r="28">
@@ -1354,10 +1354,10 @@
         <v>1</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G28" s="10" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="29">
@@ -1387,19 +1387,19 @@
         <v>1</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3250</v>
+        <v>3661</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>9750</v>
+        <v>10983.2</v>
       </c>
     </row>
     <row r="30">
@@ -1420,19 +1420,19 @@
         <v>1</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>3250</v>
+        <v>3661</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>9750</v>
+        <v>10983.2</v>
       </c>
     </row>
     <row r="31">
@@ -1453,10 +1453,10 @@
         <v>1</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>0</v>
@@ -1465,7 +1465,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="32">
@@ -1486,19 +1486,19 @@
         <v>2</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>3250</v>
+        <v>3661</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>16250</v>
+        <v>18305.4</v>
       </c>
     </row>
     <row r="33">
@@ -1519,19 +1519,19 @@
         <v>2</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>6500</v>
+        <v>7322</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>19500</v>
+        <v>21966.4</v>
       </c>
     </row>
     <row r="34">
@@ -1552,10 +1552,10 @@
         <v>1</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G34" s="10" t="n">
         <v>0</v>
@@ -1564,7 +1564,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="35">
@@ -1585,19 +1585,19 @@
         <v>2</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>6500</v>
+        <v>7322</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>19500</v>
+        <v>21966.4</v>
       </c>
     </row>
     <row r="36">
@@ -1618,10 +1618,10 @@
         <v>1</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="37">
@@ -1651,10 +1651,10 @@
         <v>2</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G37" s="7" t="n">
         <v>0</v>
@@ -1663,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
     </row>
     <row r="38">
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G38" s="10" t="n">
         <v>0</v>
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="39">
@@ -1717,19 +1717,19 @@
         <v>2</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3250</v>
+        <v>3661</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>16250</v>
+        <v>18305.4</v>
       </c>
     </row>
     <row r="40">
@@ -1750,10 +1750,10 @@
         <v>1</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="G40" s="10" t="n">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="10" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
     </row>
     <row r="41">
@@ -1783,10 +1783,10 @@
         <v>2</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>6500</v>
+        <v>7322.2</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>13000</v>
+        <v>14644.4</v>
       </c>
     </row>
     <row r="42">
@@ -1816,10 +1816,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="G42" s="10" t="n">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
     </row>
     <row r="43">
@@ -1849,19 +1849,19 @@
         <v>2</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>3299</v>
+        <v>3716</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>16494</v>
+        <v>18580.06</v>
       </c>
     </row>
     <row r="44">
@@ -1882,10 +1882,10 @@
         <v>2</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>6597.5</v>
+        <v>7432.03</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
       <c r="G44" s="10" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>13195</v>
+        <v>14864.06</v>
       </c>
     </row>
     <row r="45">
@@ -1915,10 +1915,10 @@
         <v>1</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="46">
@@ -1948,10 +1948,10 @@
         <v>2</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
       <c r="G46" s="10" t="n">
         <v>0</v>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
     </row>
     <row r="47">
@@ -1981,19 +1981,19 @@
         <v>2</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>3299</v>
+        <v>3772</v>
       </c>
       <c r="H47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>16494</v>
+        <v>18859.04</v>
       </c>
     </row>
     <row r="48">
@@ -2014,19 +2014,19 @@
         <v>2</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
       <c r="G48" s="10" t="n">
-        <v>3299</v>
+        <v>3772</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>16494</v>
+        <v>18859.04</v>
       </c>
     </row>
     <row r="49">
@@ -2047,19 +2047,19 @@
         <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>3299</v>
+        <v>3772</v>
       </c>
       <c r="H49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>9896.5</v>
+        <v>11315.52</v>
       </c>
     </row>
     <row r="50">
@@ -2080,10 +2080,10 @@
         <v>2</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
       <c r="G50" s="10" t="n">
         <v>0</v>
@@ -2092,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
     </row>
     <row r="51">
@@ -2113,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>0</v>
@@ -2125,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="52">
@@ -2146,10 +2146,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G52" s="10" t="n">
         <v>0</v>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="53">
@@ -2179,19 +2179,19 @@
         <v>2</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>13195</v>
+        <v>15087.04</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>3299</v>
+        <v>3772</v>
       </c>
       <c r="H53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>16494</v>
+        <v>18859.04</v>
       </c>
     </row>
     <row r="54">
@@ -2212,10 +2212,10 @@
         <v>3</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>19792.5</v>
+        <v>22630.56</v>
       </c>
       <c r="G54" s="10" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>19792.5</v>
+        <v>22630.56</v>
       </c>
     </row>
     <row r="55">
@@ -2245,10 +2245,10 @@
         <v>1</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="56">
@@ -2278,10 +2278,10 @@
         <v>1</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F56" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="57">
@@ -2311,10 +2311,10 @@
         <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>0</v>
@@ -2323,7 +2323,7 @@
         <v>0</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="58">
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G58" s="10" t="n">
         <v>0</v>
@@ -2356,7 +2356,7 @@
         <v>0</v>
       </c>
       <c r="I58" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="59">
@@ -2377,19 +2377,19 @@
         <v>1</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>3299</v>
+        <v>3772</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>9896.5</v>
+        <v>11315.52</v>
       </c>
     </row>
     <row r="60">
@@ -2410,10 +2410,10 @@
         <v>1</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
       <c r="G60" s="10" t="n">
         <v>0</v>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
       <c r="I60" s="10" t="n">
-        <v>6597.5</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="61">
@@ -2443,19 +2443,19 @@
         <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="62">
@@ -2476,19 +2476,19 @@
         <v>2</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="10" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="63">
@@ -2509,19 +2509,19 @@
         <v>2</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="64">
@@ -2542,19 +2542,19 @@
         <v>1</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I64" s="10" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="65">
@@ -2575,19 +2575,19 @@
         <v>2</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="66">
@@ -2608,19 +2608,19 @@
         <v>1</v>
       </c>
       <c r="E66" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="10" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="67">
@@ -2641,10 +2641,10 @@
         <v>2</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>0</v>
@@ -2653,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
     </row>
     <row r="68">
@@ -2674,19 +2674,19 @@
         <v>2</v>
       </c>
       <c r="E68" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F68" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H68" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I68" s="10" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="69">
@@ -2707,19 +2707,19 @@
         <v>1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="70">
@@ -2740,10 +2740,10 @@
         <v>1</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F70" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G70" s="10" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         <v>0</v>
       </c>
       <c r="I70" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="71">
@@ -2773,10 +2773,10 @@
         <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>0</v>
@@ -2785,7 +2785,7 @@
         <v>0</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
     </row>
     <row r="72">
@@ -2806,10 +2806,10 @@
         <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G72" s="10" t="n">
         <v>0</v>
@@ -2818,7 +2818,7 @@
         <v>0</v>
       </c>
       <c r="I72" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="73">
@@ -2839,19 +2839,19 @@
         <v>1</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F73" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G73" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H73" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="74">
@@ -2872,19 +2872,19 @@
         <v>1</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F74" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H74" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I74" s="10" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="75">
@@ -2905,19 +2905,19 @@
         <v>1</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F75" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G75" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H75" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="76">
@@ -2938,10 +2938,10 @@
         <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G76" s="10" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="I76" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="77">
@@ -2971,19 +2971,19 @@
         <v>1</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G77" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H77" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="78">
@@ -3004,19 +3004,19 @@
         <v>1</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I78" s="10" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="79">
@@ -3037,19 +3037,19 @@
         <v>2</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G79" s="7" t="n">
-        <v>6696</v>
+        <v>7656</v>
       </c>
       <c r="H79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>20088.92</v>
+        <v>22969.34</v>
       </c>
     </row>
     <row r="80">
@@ -3070,10 +3070,10 @@
         <v>1</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>0</v>
@@ -3082,7 +3082,7 @@
         <v>0</v>
       </c>
       <c r="I80" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="81">
@@ -3103,19 +3103,19 @@
         <v>2</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G81" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H81" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="82">
@@ -3136,19 +3136,19 @@
         <v>1</v>
       </c>
       <c r="E82" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H82" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I82" s="10" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="83">
@@ -3169,10 +3169,10 @@
         <v>1</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F83" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G83" s="7" t="n">
         <v>0</v>
@@ -3181,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="84">
@@ -3202,19 +3202,19 @@
         <v>2</v>
       </c>
       <c r="E84" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H84" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I84" s="10" t="n">
-        <v>16740.92</v>
+        <v>19141.34</v>
       </c>
     </row>
     <row r="85">
@@ -3235,19 +3235,19 @@
         <v>1</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G85" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H85" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I85" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="86">
@@ -3268,10 +3268,10 @@
         <v>2</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>0</v>
@@ -3280,7 +3280,7 @@
         <v>0</v>
       </c>
       <c r="I86" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
     </row>
     <row r="87">
@@ -3301,19 +3301,19 @@
         <v>2</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F87" s="7" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G87" s="7" t="n">
-        <v>6696</v>
+        <v>7656</v>
       </c>
       <c r="H87" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>20088.92</v>
+        <v>22969.34</v>
       </c>
     </row>
     <row r="88">
@@ -3334,10 +3334,10 @@
         <v>2</v>
       </c>
       <c r="E88" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>0</v>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="I88" s="10" t="n">
-        <v>13392.92</v>
+        <v>15313.34</v>
       </c>
     </row>
     <row r="89">
@@ -3367,10 +3367,10 @@
         <v>1</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F89" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G89" s="7" t="n">
         <v>0</v>
@@ -3379,7 +3379,7 @@
         <v>0</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="90">
@@ -3400,10 +3400,10 @@
         <v>1</v>
       </c>
       <c r="E90" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>0</v>
@@ -3412,7 +3412,7 @@
         <v>0</v>
       </c>
       <c r="I90" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="91">
@@ -3433,19 +3433,19 @@
         <v>1</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F91" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G91" s="7" t="n">
-        <v>3348</v>
+        <v>3828</v>
       </c>
       <c r="H91" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I91" s="7" t="n">
-        <v>10044.46</v>
+        <v>11484.67</v>
       </c>
     </row>
     <row r="92">
@@ -3466,10 +3466,10 @@
         <v>1</v>
       </c>
       <c r="E92" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>0</v>
@@ -3478,7 +3478,7 @@
         <v>0</v>
       </c>
       <c r="I92" s="10" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="93">
@@ -3499,10 +3499,10 @@
         <v>1</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
       <c r="G93" s="7" t="n">
         <v>0</v>
@@ -3511,7 +3511,7 @@
         <v>0</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>6696.46</v>
+        <v>7656.67</v>
       </c>
     </row>
     <row r="94">
@@ -3532,10 +3532,10 @@
         <v>1</v>
       </c>
       <c r="E94" s="10" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="F94" s="10" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>0</v>
@@ -3544,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="I94" s="10" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
     </row>
     <row r="95">
@@ -3565,19 +3565,19 @@
         <v>1</v>
       </c>
       <c r="E95" s="7" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="F95" s="7" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="G95" s="7" t="n">
-        <v>3348</v>
+        <v>3772</v>
       </c>
       <c r="H95" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>10044.46</v>
+        <v>11315.52</v>
       </c>
     </row>
     <row r="96">
@@ -3598,19 +3598,19 @@
         <v>1</v>
       </c>
       <c r="E96" s="10" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="G96" s="10" t="n">
-        <v>3348</v>
+        <v>3772</v>
       </c>
       <c r="H96" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I96" s="10" t="n">
-        <v>10044.46</v>
+        <v>11315.52</v>
       </c>
     </row>
     <row r="97">
@@ -3631,19 +3631,19 @@
         <v>2</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>6696.46</v>
+        <v>7543.52</v>
       </c>
       <c r="F97" s="7" t="n">
-        <v>13392.92</v>
+        <v>15087.04</v>
       </c>
       <c r="G97" s="7" t="n">
-        <v>6696</v>
+        <v>7544</v>
       </c>
       <c r="H97" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>20088.92</v>
+        <v>22631.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Oatside Pages: scope manual returns to report window (drop carry-over 22/04 +3,250) -> grand 1,496,160 reconciles with trips Excel
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
+++ b/reports/oatside-pg-2026/exports/02_Plate_DestDay_Daily.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Plate_DestDay" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plate_DestDay'!$A$4:$I$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plate_DestDay'!$A$4:$I$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I128"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-08 23:00</t>
+          <t>2026-06-09 11:47</t>
         </is>
       </c>
     </row>
@@ -579,35 +579,35 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46134</v>
+        <v>46143</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>6500</v>
+        <v>7264</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>3250</v>
+        <v>0</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>3250</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="6">
@@ -616,22 +616,22 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>7264</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>7264</v>
+        <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>7264</v>
@@ -640,21 +640,21 @@
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
@@ -682,12 +682,12 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
@@ -715,7 +715,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -724,22 +724,22 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>7264</v>
+        <v>3632</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7264</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="10">
@@ -748,7 +748,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -757,55 +757,55 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>7264</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>7264</v>
+        <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>3632</v>
+        <v>7264</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>10896</v>
+        <v>7264</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>7264</v>
+        <v>3632</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>7264</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="12">
@@ -814,12 +814,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
@@ -847,7 +847,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -876,16 +876,16 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
@@ -913,12 +913,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1008,11 +1008,11 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1054,22 +1054,22 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="20">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -1107,11 +1107,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -1173,35 +1173,35 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>14528</v>
+        <v>0</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
     </row>
     <row r="24">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -1219,22 +1219,22 @@
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="10" t="n">
         <v>7264</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>7264</v>
+        <v>3632</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>7264</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="25">
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -1305,35 +1305,35 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>7264</v>
+        <v>7168</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>7264</v>
+        <v>7168</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3632</v>
+        <v>3584</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>10896</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="28">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -1375,31 +1375,31 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>7168</v>
+        <v>14336</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="30">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -1417,55 +1417,55 @@
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="10" t="n">
         <v>7168</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>14336</v>
+        <v>7168</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>14336</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>7168</v>
+        <v>14336</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="H31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="32">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -1483,22 +1483,22 @@
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="10" t="n">
         <v>7168</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>14336</v>
+        <v>7168</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>14336</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="33">
@@ -1507,31 +1507,31 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D33" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>7168</v>
+        <v>14336</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="34">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>72-1218</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -1569,35 +1569,35 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>72-1218</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>14336</v>
+        <v>7168</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>14336</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="36">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -1627,10 +1627,10 @@
         <v>3584</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="37">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D37" s="6" t="n">
@@ -1660,24 +1660,24 @@
         <v>3584</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14336</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -1714,22 +1714,22 @@
         </is>
       </c>
       <c r="D39" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>7168</v>
+        <v>14336</v>
       </c>
       <c r="G39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="7" t="n">
         <v>3584</v>
       </c>
-      <c r="H39" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="I39" s="7" t="n">
-        <v>10752</v>
+        <v>17920</v>
       </c>
     </row>
     <row r="40">
@@ -1738,64 +1738,64 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" s="10" t="n">
         <v>7168</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>14336</v>
+        <v>7168</v>
       </c>
       <c r="G40" s="10" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="H40" s="10" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="I40" s="10" t="n">
-        <v>17920</v>
+        <v>10752</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>7168</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>7168</v>
+        <v>14336</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>3584</v>
+        <v>0</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="42">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
@@ -1837,12 +1837,12 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
@@ -1866,35 +1866,35 @@
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>7168</v>
+        <v>7264</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>14336</v>
+        <v>7264</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H44" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>14336</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="45">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -1936,64 +1936,64 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46" s="10" t="n">
         <v>7264</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G46" s="10" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H46" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>7264</v>
+        <v>7360</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>14528</v>
+        <v>7360</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>14528</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="48">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -2011,22 +2011,22 @@
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G48" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="49">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -2044,22 +2044,22 @@
         </is>
       </c>
       <c r="D49" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="50">
@@ -2068,64 +2068,64 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D51" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G51" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H51" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="52">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
@@ -2143,22 +2143,22 @@
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H52" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="53">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -2176,22 +2176,22 @@
         </is>
       </c>
       <c r="D53" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="54">
@@ -2200,12 +2200,12 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
@@ -2229,35 +2229,35 @@
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E55" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G55" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H55" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="56">
@@ -2266,12 +2266,12 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
@@ -2295,16 +2295,16 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D57" s="6" t="n">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
@@ -2341,22 +2341,22 @@
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I58" s="10" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="59">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -2374,22 +2374,22 @@
         </is>
       </c>
       <c r="D59" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>7360</v>
+        <v>0</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>3680</v>
+        <v>7360</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>11040</v>
+        <v>7360</v>
       </c>
     </row>
     <row r="60">
@@ -2398,45 +2398,45 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>7360</v>
+        <v>3680</v>
       </c>
       <c r="H60" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I60" s="10" t="n">
-        <v>7360</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D61" s="6" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
@@ -2473,22 +2473,22 @@
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="63">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -2506,22 +2506,22 @@
         </is>
       </c>
       <c r="D63" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="64">
@@ -2530,12 +2530,12 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D64" s="9" t="n">
@@ -2559,35 +2559,35 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D65" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>7360</v>
+        <v>7456</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>7360</v>
+        <v>7456</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>3680</v>
+        <v>3728</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>11040</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="66">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
@@ -2605,22 +2605,22 @@
         </is>
       </c>
       <c r="D66" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="10" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="67">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -2638,22 +2638,22 @@
         </is>
       </c>
       <c r="D67" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G67" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H67" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>14912</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="68">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C68" s="9" t="inlineStr">
@@ -2695,58 +2695,58 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D69" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E69" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F70" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0</v>
+        <v>7456</v>
       </c>
       <c r="H70" s="10" t="n">
         <v>0</v>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -2770,22 +2770,22 @@
         </is>
       </c>
       <c r="D71" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G71" s="7" t="n">
-        <v>7456</v>
+        <v>0</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="72">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C72" s="9" t="inlineStr">
@@ -2803,22 +2803,22 @@
         </is>
       </c>
       <c r="D72" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H72" s="10" t="n">
         <v>3728</v>
       </c>
       <c r="I72" s="10" t="n">
-        <v>18640</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="73">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -2860,12 +2860,12 @@
       </c>
       <c r="B74" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D74" s="9" t="n">
@@ -2881,43 +2881,43 @@
         <v>3728</v>
       </c>
       <c r="H74" s="10" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="I74" s="10" t="n">
-        <v>14912</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D75" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F75" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="7" t="n">
         <v>3728</v>
       </c>
-      <c r="H75" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="I75" s="7" t="n">
-        <v>11184</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="76">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
@@ -2935,22 +2935,22 @@
         </is>
       </c>
       <c r="D76" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H76" s="10" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="I76" s="10" t="n">
-        <v>18640</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="77">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
@@ -3025,12 +3025,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D79" s="6" t="n">
@@ -3054,16 +3054,16 @@
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D80" s="9" t="n">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -3166,22 +3166,22 @@
         </is>
       </c>
       <c r="D83" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F83" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G83" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="7" t="n">
         <v>3728</v>
       </c>
-      <c r="H83" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="I83" s="7" t="n">
-        <v>11184</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="84">
@@ -3190,64 +3190,64 @@
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H84" s="10" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="I84" s="10" t="n">
-        <v>18640</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D85" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E85" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G85" s="7" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H85" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I85" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="86">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B86" s="9" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C86" s="9" t="inlineStr">
@@ -3265,22 +3265,22 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E86" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H86" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I86" s="10" t="n">
-        <v>14912</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="87">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="B88" s="9" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C88" s="9" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D89" s="6" t="n">
@@ -3384,16 +3384,16 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
       <c r="B90" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D90" s="9" t="n">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -3430,22 +3430,22 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E91" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F91" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G91" s="7" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H91" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I91" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="92">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="B92" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C92" s="9" t="inlineStr">
@@ -3463,22 +3463,22 @@
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H92" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I92" s="10" t="n">
-        <v>14912</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="93">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -3496,22 +3496,22 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G93" s="7" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H93" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="94">
@@ -3520,12 +3520,12 @@
       </c>
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D94" s="9" t="n">
@@ -3549,35 +3549,35 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E95" s="7" t="n">
         <v>7456</v>
       </c>
       <c r="F95" s="7" t="n">
-        <v>14912</v>
+        <v>7456</v>
       </c>
       <c r="G95" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="H95" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>14912</v>
+        <v>11184</v>
       </c>
     </row>
     <row r="96">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C96" s="9" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -3652,64 +3652,64 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D98" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E98" s="10" t="n">
         <v>7456</v>
       </c>
       <c r="F98" s="10" t="n">
-        <v>7456</v>
+        <v>14912</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>3728</v>
+        <v>0</v>
       </c>
       <c r="H98" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I98" s="10" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n">
-        <v>46167</v>
+        <v>46168</v>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E99" s="7" t="n">
-        <v>7456</v>
+        <v>7360</v>
       </c>
       <c r="F99" s="7" t="n">
-        <v>14912</v>
+        <v>7360</v>
       </c>
       <c r="G99" s="7" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H99" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I99" s="7" t="n">
-        <v>14912</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="100">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr">
@@ -3727,22 +3727,22 @@
         </is>
       </c>
       <c r="D100" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E100" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F100" s="10" t="n">
-        <v>7360</v>
+        <v>0</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>3680</v>
+        <v>7360</v>
       </c>
       <c r="H100" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I100" s="10" t="n">
-        <v>11040</v>
+        <v>7360</v>
       </c>
     </row>
     <row r="101">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8005</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -3760,22 +3760,22 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F101" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="G101" s="7" t="n">
-        <v>7360</v>
+        <v>3680</v>
       </c>
       <c r="H101" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>7360</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="102">
@@ -3784,7 +3784,7 @@
       </c>
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>71-8005</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C102" s="9" t="inlineStr">
@@ -3817,45 +3817,45 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F103" s="7" t="n">
-        <v>7360</v>
+        <v>0</v>
       </c>
       <c r="G103" s="7" t="n">
-        <v>3680</v>
+        <v>7360</v>
       </c>
       <c r="H103" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>11040</v>
+        <v>7360</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D104" s="9" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -3892,22 +3892,22 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F105" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="G105" s="7" t="n">
-        <v>7360</v>
+        <v>3680</v>
       </c>
       <c r="H105" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>7360</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="106">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B106" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -3982,12 +3982,12 @@
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D108" s="9" t="n">
@@ -4011,16 +4011,16 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D109" s="6" t="n">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C110" s="9" t="inlineStr">
@@ -4057,22 +4057,22 @@
         </is>
       </c>
       <c r="D110" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F110" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G110" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H110" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I110" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="111">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="B112" s="9" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C112" s="9" t="inlineStr">
@@ -4123,22 +4123,22 @@
         </is>
       </c>
       <c r="D112" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E112" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F112" s="10" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G112" s="10" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H112" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I112" s="10" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="113">
@@ -4147,12 +4147,12 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D113" s="6" t="n">
@@ -4176,35 +4176,35 @@
     </row>
     <row r="114">
       <c r="A114" s="8" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B114" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D114" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E114" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F114" s="10" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G114" s="10" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H114" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I114" s="10" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="115">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C116" s="9" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -4312,64 +4312,64 @@
       </c>
       <c r="B118" s="9" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D118" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E118" s="10" t="n">
         <v>7360</v>
       </c>
       <c r="F118" s="10" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G118" s="10" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H118" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I118" s="10" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D119" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E119" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="F119" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>3680</v>
+        <v>3632</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I119" s="7" t="n">
-        <v>11040</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="120">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C120" s="9" t="inlineStr">
@@ -4387,22 +4387,22 @@
         </is>
       </c>
       <c r="D120" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E120" s="10" t="n">
         <v>7264</v>
       </c>
       <c r="F120" s="10" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G120" s="10" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H120" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I120" s="10" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="121">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -4420,22 +4420,22 @@
         </is>
       </c>
       <c r="D121" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F121" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="122">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C122" s="9" t="inlineStr">
@@ -4477,45 +4477,45 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D123" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E123" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F123" s="7" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I123" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D124" s="9" t="n">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
@@ -4552,22 +4552,22 @@
         </is>
       </c>
       <c r="D125" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E125" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F125" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G125" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H125" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I125" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="126">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B126" s="9" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C126" s="9" t="inlineStr">
@@ -4609,12 +4609,12 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D127" s="6" t="n">
@@ -4636,41 +4636,8 @@
         <v>10896</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B128" s="9" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C128" s="9" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D128" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E128" s="10" t="n">
-        <v>7264</v>
-      </c>
-      <c r="F128" s="10" t="n">
-        <v>7264</v>
-      </c>
-      <c r="G128" s="10" t="n">
-        <v>3632</v>
-      </c>
-      <c r="H128" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" s="10" t="n">
-        <v>10896</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:I128"/>
+  <autoFilter ref="A4:I127"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>

</xml_diff>